<commit_message>
etapa 3 básico OK :) YUPIII
</commit_message>
<xml_diff>
--- a/output/_temp/etapa_3_clasificacion/Cierre de OT Turno 16.04 al 22.04.xlsx
+++ b/output/_temp/etapa_3_clasificacion/Cierre de OT Turno 16.04 al 22.04.xlsx
@@ -2423,11 +2423,7 @@
         <f>IF(H7="TT","TRABAJO TERMINADO",IF(H7="MI","TRABAJO NO TERMINADO",""))</f>
         <v/>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>TT</t>
-        </is>
-      </c>
+      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="7">
         <f>IF(B7="", G7, IF(G7="", LEFT(B7,45), IF(45-LEN(G7)-2&lt;=0, G7, LEFT(B7,45-LEN(G7)-2)&amp;", "&amp;G7)))</f>
         <v/>

</xml_diff>